<commit_message>
Windows: Increase number of peaks
</commit_message>
<xml_diff>
--- a/Data-Examples/Valence Band/Au_Valence.xlsx
+++ b/Data-Examples/Valence Band/Au_Valence.xlsx
@@ -478,7 +478,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5610225" cy="3990975"/>
+    <ext cx="5591175" cy="3990975"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1106,37 +1106,37 @@
         <v>1488.96</v>
       </c>
       <c r="I2" t="n">
-        <v>1.84</v>
+        <v>1.824685903352903</v>
       </c>
       <c r="J2" t="n">
-        <v>2.33</v>
+        <v>2.26</v>
       </c>
       <c r="K2" t="n">
-        <v>-1.2</v>
+        <v>-1.04</v>
       </c>
       <c r="L2" t="n">
         <v>-1.92</v>
       </c>
       <c r="M2" t="n">
-        <v>-46702.64479999999</v>
+        <v>-44700.71587878797</v>
       </c>
       <c r="N2" t="n">
-        <v>2.58</v>
+        <v>2.53</v>
       </c>
       <c r="O2" t="n">
-        <v>9519.950000000001</v>
+        <v>8949.08</v>
       </c>
       <c r="P2" t="n">
         <v>-1.92</v>
       </c>
       <c r="Q2" t="n">
-        <v>28.6016</v>
+        <v>16.3971431578947</v>
       </c>
       <c r="R2" t="n">
-        <v>-0.72</v>
+        <v>-0.52</v>
       </c>
       <c r="S2" t="n">
-        <v>100.41</v>
+        <v>121.394</v>
       </c>
       <c r="X2" s="21" t="inlineStr">
         <is>
@@ -1150,89 +1150,49 @@
       </c>
       <c r="Z2" s="22" t="inlineStr">
         <is>
-          <t>1.84</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="AA2" s="22" t="inlineStr">
         <is>
-          <t>2.33</t>
+          <t>2.26</t>
         </is>
       </c>
       <c r="AB2" s="22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="AC2" s="22" t="inlineStr">
         <is>
-          <t>-1.2</t>
+          <t>-1.04</t>
         </is>
       </c>
       <c r="AD2" s="22" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="AE2" s="22" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AF2" s="22" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AG2" s="22" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AH2" s="22" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="AI2" s="22" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="AJ2" s="22" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="AF2" s="22" t="inlineStr"/>
+      <c r="AG2" s="22" t="inlineStr"/>
+      <c r="AH2" s="22" t="inlineStr"/>
+      <c r="AI2" s="22" t="inlineStr"/>
+      <c r="AJ2" s="22" t="inlineStr"/>
       <c r="AK2" s="22" t="inlineStr">
         <is>
           <t>VBM</t>
         </is>
       </c>
-      <c r="AL2" s="22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AM2" s="22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AN2" s="22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AO2" s="22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AP2" s="22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="AL2" s="22" t="inlineStr"/>
+      <c r="AM2" s="22" t="inlineStr"/>
+      <c r="AN2" s="22" t="inlineStr"/>
+      <c r="AO2" s="22" t="inlineStr"/>
+      <c r="AP2" s="22" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1251,68 +1211,36 @@
         <v>-1.748282828282828</v>
       </c>
       <c r="M3" t="n">
-        <v>-44559.71065858586</v>
+        <v>-42637.99447076839</v>
       </c>
       <c r="N3" t="n">
-        <v>2.53</v>
+        <v>2.48</v>
       </c>
       <c r="O3" t="n">
-        <v>8949.08</v>
+        <v>8185.47</v>
       </c>
       <c r="P3" t="n">
         <v>-1.748282828282828</v>
       </c>
       <c r="Q3" t="n">
-        <v>38.0494787878788</v>
+        <v>28.56040727272725</v>
       </c>
       <c r="R3" t="n">
-        <v>-0.77</v>
+        <v>-0.57</v>
       </c>
       <c r="S3" t="n">
-        <v>90.51000000000001</v>
+        <v>116.229</v>
       </c>
       <c r="X3" s="23" t="inlineStr"/>
       <c r="Y3" s="24" t="inlineStr"/>
-      <c r="Z3" s="24" t="inlineStr">
-        <is>
-          <t>-1.92:15.08</t>
-        </is>
-      </c>
-      <c r="AA3" s="24" t="inlineStr">
-        <is>
-          <t>1:1e7</t>
-        </is>
-      </c>
-      <c r="AB3" s="24" t="inlineStr">
-        <is>
-          <t>0.3:3.7</t>
-        </is>
-      </c>
-      <c r="AC3" s="24" t="inlineStr">
-        <is>
-          <t>5:80</t>
-        </is>
-      </c>
-      <c r="AD3" s="24" t="inlineStr">
-        <is>
-          <t>1:1e7</t>
-        </is>
-      </c>
-      <c r="AE3" s="24" t="inlineStr">
-        <is>
-          <t>0.3:3</t>
-        </is>
-      </c>
-      <c r="AF3" s="24" t="inlineStr">
-        <is>
-          <t>0.3:3</t>
-        </is>
-      </c>
-      <c r="AG3" s="24" t="inlineStr">
-        <is>
-          <t>0.01:2</t>
-        </is>
-      </c>
+      <c r="Z3" s="24" t="inlineStr"/>
+      <c r="AA3" s="24" t="inlineStr"/>
+      <c r="AB3" s="24" t="inlineStr"/>
+      <c r="AC3" s="24" t="inlineStr"/>
+      <c r="AD3" s="24" t="inlineStr"/>
+      <c r="AE3" s="24" t="inlineStr"/>
+      <c r="AF3" s="24" t="inlineStr"/>
+      <c r="AG3" s="24" t="inlineStr"/>
       <c r="AH3" s="24" t="inlineStr"/>
       <c r="AI3" s="24" t="inlineStr"/>
       <c r="AJ3" s="24" t="inlineStr"/>
@@ -1340,25 +1268,25 @@
         <v>-1.576565656565657</v>
       </c>
       <c r="M4" t="n">
-        <v>-42416.77651717172</v>
+        <v>-40575.27306274879</v>
       </c>
       <c r="N4" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="O4" t="n">
-        <v>8185.47</v>
+        <v>7569.66</v>
       </c>
       <c r="P4" t="n">
         <v>-1.576565656565657</v>
       </c>
       <c r="Q4" t="n">
-        <v>47.49735757575759</v>
+        <v>40.72367138755979</v>
       </c>
       <c r="R4" t="n">
-        <v>-0.82</v>
+        <v>-0.62</v>
       </c>
       <c r="S4" t="n">
-        <v>87.19</v>
+        <v>105.313</v>
       </c>
       <c r="X4" s="25" t="inlineStr">
         <is>
@@ -1383,25 +1311,25 @@
         <v>-1.404848484848485</v>
       </c>
       <c r="M5" t="n">
-        <v>-40273.84237575758</v>
+        <v>-38512.55165472919</v>
       </c>
       <c r="N5" t="n">
-        <v>2.43</v>
+        <v>2.38</v>
       </c>
       <c r="O5" t="n">
-        <v>7569.66</v>
+        <v>6806.91</v>
       </c>
       <c r="P5" t="n">
         <v>-1.404848484848485</v>
       </c>
       <c r="Q5" t="n">
-        <v>56.94523636363637</v>
+        <v>52.88693550239233</v>
       </c>
       <c r="R5" t="n">
-        <v>-0.87</v>
+        <v>-0.67</v>
       </c>
       <c r="S5" t="n">
-        <v>99.09999999999999</v>
+        <v>119.027</v>
       </c>
     </row>
     <row r="6">
@@ -1421,25 +1349,25 @@
         <v>-1.233131313131313</v>
       </c>
       <c r="M6" t="n">
-        <v>-38130.90823434343</v>
+        <v>-36449.8302467096</v>
       </c>
       <c r="N6" t="n">
-        <v>2.38</v>
+        <v>2.33</v>
       </c>
       <c r="O6" t="n">
-        <v>6806.91</v>
+        <v>6293.8</v>
       </c>
       <c r="P6" t="n">
         <v>-1.233131313131313</v>
       </c>
       <c r="Q6" t="n">
-        <v>66.39311515151516</v>
+        <v>65.05019961722488</v>
       </c>
       <c r="R6" t="n">
-        <v>-0.92</v>
+        <v>-0.72</v>
       </c>
       <c r="S6" t="n">
-        <v>74.77</v>
+        <v>100.411</v>
       </c>
     </row>
     <row r="7">
@@ -1459,25 +1387,25 @@
         <v>-1.061414141414141</v>
       </c>
       <c r="M7" t="n">
-        <v>-35987.97409292929</v>
+        <v>-34387.10883869001</v>
       </c>
       <c r="N7" t="n">
-        <v>2.33</v>
+        <v>2.28</v>
       </c>
       <c r="O7" t="n">
-        <v>6293.8</v>
+        <v>5595.72</v>
       </c>
       <c r="P7" t="n">
         <v>-1.061414141414141</v>
       </c>
       <c r="Q7" t="n">
-        <v>75.84099393939394</v>
+        <v>77.21346373205742</v>
       </c>
       <c r="R7" t="n">
-        <v>-0.97</v>
+        <v>-0.77</v>
       </c>
       <c r="S7" t="n">
-        <v>81.36</v>
+        <v>90.5068</v>
       </c>
     </row>
     <row r="8">
@@ -1497,25 +1425,25 @@
         <v>-0.8896969696969697</v>
       </c>
       <c r="M8" t="n">
-        <v>-33845.03995151515</v>
+        <v>-32324.38743067041</v>
       </c>
       <c r="N8" t="n">
-        <v>2.28</v>
+        <v>2.23</v>
       </c>
       <c r="O8" t="n">
-        <v>5595.72</v>
+        <v>5029.14</v>
       </c>
       <c r="P8" t="n">
         <v>-0.8896969696969697</v>
       </c>
       <c r="Q8" t="n">
-        <v>85.28887272727275</v>
+        <v>89.37672784688996</v>
       </c>
       <c r="R8" t="n">
-        <v>-1.02</v>
+        <v>-0.82</v>
       </c>
       <c r="S8" t="n">
-        <v>76.68000000000001</v>
+        <v>87.19199999999999</v>
       </c>
     </row>
     <row r="9">
@@ -1535,25 +1463,25 @@
         <v>-0.7179797979797979</v>
       </c>
       <c r="M9" t="n">
-        <v>-31702.10581010101</v>
+        <v>-30261.66602265082</v>
       </c>
       <c r="N9" t="n">
-        <v>2.23</v>
+        <v>2.18</v>
       </c>
       <c r="O9" t="n">
-        <v>5029.14</v>
+        <v>4547.03</v>
       </c>
       <c r="P9" t="n">
         <v>-0.7179797979797979</v>
       </c>
       <c r="Q9" t="n">
-        <v>94.73675151515152</v>
+        <v>101.5399919617225</v>
       </c>
       <c r="R9" t="n">
-        <v>-1.07</v>
+        <v>-0.87</v>
       </c>
       <c r="S9" t="n">
-        <v>68.08</v>
+        <v>99.09950000000001</v>
       </c>
     </row>
     <row r="10">
@@ -1573,25 +1501,25 @@
         <v>-0.5462626262626262</v>
       </c>
       <c r="M10" t="n">
-        <v>-29559.17166868687</v>
+        <v>-28198.94461463122</v>
       </c>
       <c r="N10" t="n">
-        <v>2.18</v>
+        <v>2.13</v>
       </c>
       <c r="O10" t="n">
-        <v>4547.03</v>
+        <v>3972.79</v>
       </c>
       <c r="P10" t="n">
         <v>-0.5462626262626262</v>
       </c>
       <c r="Q10" t="n">
-        <v>104.1846303030303</v>
+        <v>113.703256076555</v>
       </c>
       <c r="R10" t="n">
-        <v>-1.12</v>
+        <v>-0.92</v>
       </c>
       <c r="S10" t="n">
-        <v>68.22</v>
+        <v>74.7679</v>
       </c>
     </row>
     <row r="11">
@@ -1611,25 +1539,25 @@
         <v>-0.3745454545454545</v>
       </c>
       <c r="M11" t="n">
-        <v>-27416.23752727273</v>
+        <v>-26136.22320661163</v>
       </c>
       <c r="N11" t="n">
-        <v>2.13</v>
+        <v>2.08</v>
       </c>
       <c r="O11" t="n">
-        <v>3972.79</v>
+        <v>3563.71</v>
       </c>
       <c r="P11" t="n">
         <v>-0.3745454545454545</v>
       </c>
       <c r="Q11" t="n">
-        <v>113.6325090909091</v>
+        <v>125.8665201913876</v>
       </c>
       <c r="R11" t="n">
-        <v>-1.17</v>
+        <v>-0.97</v>
       </c>
       <c r="S11" t="n">
-        <v>66.7</v>
+        <v>81.3574</v>
       </c>
     </row>
     <row r="12">
@@ -1649,19 +1577,19 @@
         <v>-0.2028282828282828</v>
       </c>
       <c r="M12" t="n">
-        <v>-25273.30338585858</v>
+        <v>-24073.50179859203</v>
       </c>
       <c r="P12" t="n">
         <v>-0.2028282828282828</v>
       </c>
       <c r="Q12" t="n">
-        <v>123.0803878787879</v>
+        <v>138.0297843062201</v>
       </c>
       <c r="R12" t="n">
-        <v>-1.22</v>
+        <v>-1.02</v>
       </c>
       <c r="S12" t="n">
-        <v>71</v>
+        <v>76.6784</v>
       </c>
     </row>
     <row r="13">
@@ -1681,19 +1609,19 @@
         <v>-0.03111111111111109</v>
       </c>
       <c r="M13" t="n">
-        <v>-23130.36924444444</v>
+        <v>-22010.78039057244</v>
       </c>
       <c r="P13" t="n">
         <v>-0.03111111111111109</v>
       </c>
       <c r="Q13" t="n">
-        <v>132.5282666666667</v>
+        <v>150.1930484210527</v>
       </c>
       <c r="R13" t="n">
-        <v>-1.27</v>
+        <v>-1.07</v>
       </c>
       <c r="S13" t="n">
-        <v>61.73</v>
+        <v>68.0821</v>
       </c>
     </row>
     <row r="14">
@@ -1713,19 +1641,19 @@
         <v>0.1406060606060606</v>
       </c>
       <c r="M14" t="n">
-        <v>-20987.4351030303</v>
+        <v>-19948.05898255284</v>
       </c>
       <c r="P14" t="n">
         <v>0.1406060606060606</v>
       </c>
       <c r="Q14" t="n">
-        <v>141.9761454545455</v>
+        <v>162.3563125358852</v>
       </c>
       <c r="R14" t="n">
-        <v>-1.32</v>
+        <v>-1.12</v>
       </c>
       <c r="S14" t="n">
-        <v>68.23</v>
+        <v>68.2179</v>
       </c>
     </row>
     <row r="15">
@@ -1745,19 +1673,19 @@
         <v>0.3123232323232323</v>
       </c>
       <c r="M15" t="n">
-        <v>-18844.50096161616</v>
+        <v>-17885.33757453325</v>
       </c>
       <c r="P15" t="n">
         <v>0.3123232323232323</v>
       </c>
       <c r="Q15" t="n">
-        <v>151.4240242424243</v>
+        <v>174.5195766507178</v>
       </c>
       <c r="R15" t="n">
-        <v>-1.37</v>
+        <v>-1.17</v>
       </c>
       <c r="S15" t="n">
-        <v>62.69</v>
+        <v>66.70440000000001</v>
       </c>
     </row>
     <row r="16">
@@ -1777,19 +1705,19 @@
         <v>0.484040404040404</v>
       </c>
       <c r="M16" t="n">
-        <v>-16701.56682020202</v>
+        <v>-15822.61616651366</v>
       </c>
       <c r="P16" t="n">
         <v>0.484040404040404</v>
       </c>
       <c r="Q16" t="n">
-        <v>160.871903030303</v>
+        <v>186.6828407655503</v>
       </c>
       <c r="R16" t="n">
-        <v>-1.42</v>
+        <v>-1.22</v>
       </c>
       <c r="S16" t="n">
-        <v>49.75</v>
+        <v>70.9995</v>
       </c>
     </row>
     <row r="17">
@@ -1809,19 +1737,19 @@
         <v>0.6557575757575758</v>
       </c>
       <c r="M17" t="n">
-        <v>-14558.63267878788</v>
+        <v>-13759.89475849406</v>
       </c>
       <c r="P17" t="n">
         <v>0.6557575757575758</v>
       </c>
       <c r="Q17" t="n">
-        <v>170.3197818181818</v>
+        <v>198.8461048803829</v>
       </c>
       <c r="R17" t="n">
-        <v>-1.47</v>
+        <v>-1.27</v>
       </c>
       <c r="S17" t="n">
-        <v>49.98</v>
+        <v>61.7336</v>
       </c>
     </row>
     <row r="18">
@@ -1841,19 +1769,19 @@
         <v>0.8274747474747475</v>
       </c>
       <c r="M18" t="n">
-        <v>-12415.69853737374</v>
+        <v>-11697.17335047447</v>
       </c>
       <c r="P18" t="n">
         <v>0.8274747474747475</v>
       </c>
       <c r="Q18" t="n">
-        <v>179.7676606060606</v>
+        <v>211.0093689952154</v>
       </c>
       <c r="R18" t="n">
-        <v>-1.52</v>
+        <v>-1.32</v>
       </c>
       <c r="S18" t="n">
-        <v>59.53</v>
+        <v>68.2252</v>
       </c>
     </row>
     <row r="19">
@@ -1873,19 +1801,19 @@
         <v>0.9991919191919192</v>
       </c>
       <c r="M19" t="n">
-        <v>-10272.7643959596</v>
+        <v>-9634.451942454873</v>
       </c>
       <c r="P19" t="n">
         <v>0.9991919191919192</v>
       </c>
       <c r="Q19" t="n">
-        <v>189.2155393939394</v>
+        <v>223.1726331100479</v>
       </c>
       <c r="R19" t="n">
-        <v>-1.57</v>
+        <v>-1.37</v>
       </c>
       <c r="S19" t="n">
-        <v>40.8</v>
+        <v>62.6902</v>
       </c>
     </row>
     <row r="20">
@@ -1905,19 +1833,19 @@
         <v>1.170909090909091</v>
       </c>
       <c r="M20" t="n">
-        <v>-8129.830254545453</v>
+        <v>-7571.730534435277</v>
       </c>
       <c r="P20" t="n">
         <v>1.170909090909091</v>
       </c>
       <c r="Q20" t="n">
-        <v>198.6634181818182</v>
+        <v>235.3358972248805</v>
       </c>
       <c r="R20" t="n">
-        <v>-1.62</v>
+        <v>-1.42</v>
       </c>
       <c r="S20" t="n">
-        <v>50.75</v>
+        <v>49.7465</v>
       </c>
     </row>
     <row r="21">
@@ -1937,13 +1865,19 @@
         <v>1.342626262626263</v>
       </c>
       <c r="M21" t="n">
-        <v>-5986.896113131312</v>
+        <v>-5509.009126415684</v>
       </c>
       <c r="P21" t="n">
         <v>1.342626262626263</v>
       </c>
       <c r="Q21" t="n">
-        <v>208.111296969697</v>
+        <v>247.499161339713</v>
+      </c>
+      <c r="R21" t="n">
+        <v>-1.47</v>
+      </c>
+      <c r="S21" t="n">
+        <v>49.9803</v>
       </c>
     </row>
     <row r="22">
@@ -1963,13 +1897,13 @@
         <v>1.514343434343434</v>
       </c>
       <c r="M22" t="n">
-        <v>-3843.96197171717</v>
+        <v>-3446.287718396088</v>
       </c>
       <c r="P22" t="n">
         <v>1.514343434343434</v>
       </c>
       <c r="Q22" t="n">
-        <v>217.5591757575758</v>
+        <v>259.6624254545455</v>
       </c>
     </row>
     <row r="23">
@@ -1989,13 +1923,13 @@
         <v>1.686060606060606</v>
       </c>
       <c r="M23" t="n">
-        <v>-1701.027830303028</v>
+        <v>-1383.566310376493</v>
       </c>
       <c r="P23" t="n">
         <v>1.686060606060606</v>
       </c>
       <c r="Q23" t="n">
-        <v>227.0070545454546</v>
+        <v>271.8256895693781</v>
       </c>
     </row>
     <row r="24">
@@ -2015,13 +1949,13 @@
         <v>1.857777777777778</v>
       </c>
       <c r="M24" t="n">
-        <v>441.9063111111136</v>
+        <v>679.1550976431026</v>
       </c>
       <c r="P24" t="n">
         <v>1.857777777777778</v>
       </c>
       <c r="Q24" t="n">
-        <v>236.4549333333333</v>
+        <v>283.9889536842106</v>
       </c>
     </row>
     <row r="25">
@@ -2041,13 +1975,13 @@
         <v>2.029494949494949</v>
       </c>
       <c r="M25" t="n">
-        <v>2584.840452525255</v>
+        <v>2741.876505662694</v>
       </c>
       <c r="P25" t="n">
         <v>2.029494949494949</v>
       </c>
       <c r="Q25" t="n">
-        <v>245.9028121212122</v>
+        <v>296.1522177990432</v>
       </c>
     </row>
     <row r="26">
@@ -2067,13 +2001,13 @@
         <v>2.201212121212121</v>
       </c>
       <c r="M26" t="n">
-        <v>4727.774593939397</v>
+        <v>4804.59791368229</v>
       </c>
       <c r="P26" t="n">
         <v>2.201212121212121</v>
       </c>
       <c r="Q26" t="n">
-        <v>255.3506909090909</v>
+        <v>308.3154819138757</v>
       </c>
     </row>
     <row r="27">
@@ -2093,13 +2027,13 @@
         <v>2.372929292929292</v>
       </c>
       <c r="M27" t="n">
-        <v>6870.708735353532</v>
+        <v>6867.319321701878</v>
       </c>
       <c r="P27" t="n">
         <v>2.372929292929292</v>
       </c>
       <c r="Q27" t="n">
-        <v>264.7985696969697</v>
+        <v>320.4787460287082</v>
       </c>
     </row>
     <row r="28">
@@ -2119,13 +2053,13 @@
         <v>2.544646464646465</v>
       </c>
       <c r="M28" t="n">
-        <v>9013.642876767677</v>
+        <v>8930.040729721481</v>
       </c>
       <c r="P28" t="n">
         <v>2.544646464646465</v>
       </c>
       <c r="Q28" t="n">
-        <v>274.2464484848485</v>
+        <v>332.6420101435408</v>
       </c>
     </row>
     <row r="29">
@@ -2145,13 +2079,13 @@
         <v>2.716363636363637</v>
       </c>
       <c r="M29" t="n">
-        <v>11156.57701818183</v>
+        <v>10992.76213774108</v>
       </c>
       <c r="P29" t="n">
         <v>2.716363636363637</v>
       </c>
       <c r="Q29" t="n">
-        <v>283.6943272727273</v>
+        <v>344.8052742583734</v>
       </c>
     </row>
     <row r="30">
@@ -2171,13 +2105,13 @@
         <v>2.888080808080808</v>
       </c>
       <c r="M30" t="n">
-        <v>13299.51115959596</v>
+        <v>13055.48354576067</v>
       </c>
       <c r="P30" t="n">
         <v>2.888080808080808</v>
       </c>
       <c r="Q30" t="n">
-        <v>293.1422060606061</v>
+        <v>356.9685383732059</v>
       </c>
     </row>
     <row r="31">
@@ -2197,13 +2131,13 @@
         <v>3.059797979797979</v>
       </c>
       <c r="M31" t="n">
-        <v>15442.4453010101</v>
+        <v>15118.20495378026</v>
       </c>
       <c r="P31" t="n">
         <v>3.059797979797979</v>
       </c>
       <c r="Q31" t="n">
-        <v>302.5900848484848</v>
+        <v>369.1318024880384</v>
       </c>
     </row>
     <row r="32">
@@ -2223,13 +2157,13 @@
         <v>3.231515151515151</v>
       </c>
       <c r="M32" t="n">
-        <v>17585.37944242425</v>
+        <v>17180.92636179985</v>
       </c>
       <c r="P32" t="n">
         <v>3.231515151515151</v>
       </c>
       <c r="Q32" t="n">
-        <v>312.0379636363637</v>
+        <v>381.295066602871</v>
       </c>
     </row>
     <row r="33">
@@ -2249,13 +2183,13 @@
         <v>3.403232323232324</v>
       </c>
       <c r="M33" t="n">
-        <v>19728.31358383839</v>
+        <v>19243.64776981945</v>
       </c>
       <c r="P33" t="n">
         <v>3.403232323232324</v>
       </c>
       <c r="Q33" t="n">
-        <v>321.4858424242425</v>
+        <v>393.4583307177036</v>
       </c>
     </row>
     <row r="34">
@@ -2275,13 +2209,13 @@
         <v>3.574949494949495</v>
       </c>
       <c r="M34" t="n">
-        <v>21871.24772525252</v>
+        <v>21306.36917783905</v>
       </c>
       <c r="P34" t="n">
         <v>3.574949494949495</v>
       </c>
       <c r="Q34" t="n">
-        <v>330.9337212121212</v>
+        <v>405.6215948325361</v>
       </c>
     </row>
     <row r="35">
@@ -2301,13 +2235,13 @@
         <v>3.746666666666666</v>
       </c>
       <c r="M35" t="n">
-        <v>24014.18186666666</v>
+        <v>23369.09058585864</v>
       </c>
       <c r="P35" t="n">
         <v>3.746666666666666</v>
       </c>
       <c r="Q35" t="n">
-        <v>340.3816</v>
+        <v>417.7848589473685</v>
       </c>
     </row>
     <row r="36">
@@ -2327,13 +2261,13 @@
         <v>3.918383838383838</v>
       </c>
       <c r="M36" t="n">
-        <v>26157.11600808081</v>
+        <v>25431.81199387824</v>
       </c>
       <c r="P36" t="n">
         <v>3.918383838383838</v>
       </c>
       <c r="Q36" t="n">
-        <v>349.8294787878788</v>
+        <v>429.9481230622011</v>
       </c>
     </row>
     <row r="37">
@@ -2353,13 +2287,13 @@
         <v>4.09010101010101</v>
       </c>
       <c r="M37" t="n">
-        <v>28300.05014949496</v>
+        <v>27494.53340189784</v>
       </c>
       <c r="P37" t="n">
         <v>4.09010101010101</v>
       </c>
       <c r="Q37" t="n">
-        <v>359.2773575757576</v>
+        <v>442.1113871770337</v>
       </c>
     </row>
     <row r="38">
@@ -2379,13 +2313,13 @@
         <v>4.261818181818182</v>
       </c>
       <c r="M38" t="n">
-        <v>30442.98429090909</v>
+        <v>29557.25480991743</v>
       </c>
       <c r="P38" t="n">
         <v>4.261818181818182</v>
       </c>
       <c r="Q38" t="n">
-        <v>368.7252363636364</v>
+        <v>454.2746512918662</v>
       </c>
     </row>
     <row r="39">
@@ -2405,13 +2339,13 @@
         <v>4.433535353535353</v>
       </c>
       <c r="M39" t="n">
-        <v>32585.91843232323</v>
+        <v>31619.97621793701</v>
       </c>
       <c r="P39" t="n">
         <v>4.433535353535353</v>
       </c>
       <c r="Q39" t="n">
-        <v>378.1731151515152</v>
+        <v>466.4379154066987</v>
       </c>
     </row>
     <row r="40">
@@ -2431,13 +2365,13 @@
         <v>4.605252525252525</v>
       </c>
       <c r="M40" t="n">
-        <v>34728.85257373737</v>
+        <v>33682.69762595661</v>
       </c>
       <c r="P40" t="n">
         <v>4.605252525252525</v>
       </c>
       <c r="Q40" t="n">
-        <v>387.620993939394</v>
+        <v>478.6011795215313</v>
       </c>
     </row>
     <row r="41">
@@ -2457,13 +2391,13 @@
         <v>4.776969696969697</v>
       </c>
       <c r="M41" t="n">
-        <v>36871.78671515152</v>
+        <v>35745.41903397621</v>
       </c>
       <c r="P41" t="n">
         <v>4.776969696969697</v>
       </c>
       <c r="Q41" t="n">
-        <v>397.0688727272728</v>
+        <v>490.7644436363639</v>
       </c>
     </row>
     <row r="42">
@@ -2483,13 +2417,13 @@
         <v>4.948686868686869</v>
       </c>
       <c r="M42" t="n">
-        <v>39014.72085656566</v>
+        <v>37808.1404419958</v>
       </c>
       <c r="P42" t="n">
         <v>4.948686868686869</v>
       </c>
       <c r="Q42" t="n">
-        <v>406.5167515151516</v>
+        <v>502.9277077511964</v>
       </c>
     </row>
     <row r="43">
@@ -2509,13 +2443,13 @@
         <v>5.12040404040404</v>
       </c>
       <c r="M43" t="n">
-        <v>41157.6549979798</v>
+        <v>39870.8618500154</v>
       </c>
       <c r="P43" t="n">
         <v>5.12040404040404</v>
       </c>
       <c r="Q43" t="n">
-        <v>415.9646303030303</v>
+        <v>515.0909718660289</v>
       </c>
     </row>
     <row r="44">
@@ -2535,13 +2469,13 @@
         <v>5.292121212121212</v>
       </c>
       <c r="M44" t="n">
-        <v>43300.58913939394</v>
+        <v>41933.583258035</v>
       </c>
       <c r="P44" t="n">
         <v>5.292121212121212</v>
       </c>
       <c r="Q44" t="n">
-        <v>425.4125090909091</v>
+        <v>527.2542359808615</v>
       </c>
     </row>
     <row r="45">
@@ -2561,13 +2495,13 @@
         <v>5.463838383838384</v>
       </c>
       <c r="M45" t="n">
-        <v>45443.52328080809</v>
+        <v>43996.3046660546</v>
       </c>
       <c r="P45" t="n">
         <v>5.463838383838384</v>
       </c>
       <c r="Q45" t="n">
-        <v>434.8603878787879</v>
+        <v>539.4175000956941</v>
       </c>
     </row>
     <row r="46">
@@ -2587,13 +2521,13 @@
         <v>5.635555555555555</v>
       </c>
       <c r="M46" t="n">
-        <v>47586.45742222223</v>
+        <v>46059.02607407418</v>
       </c>
       <c r="P46" t="n">
         <v>5.635555555555555</v>
       </c>
       <c r="Q46" t="n">
-        <v>444.3082666666667</v>
+        <v>551.5807642105266</v>
       </c>
     </row>
     <row r="47">
@@ -2613,13 +2547,13 @@
         <v>5.807272727272727</v>
       </c>
       <c r="M47" t="n">
-        <v>49729.39156363637</v>
+        <v>48121.74748209376</v>
       </c>
       <c r="P47" t="n">
         <v>5.807272727272727</v>
       </c>
       <c r="Q47" t="n">
-        <v>453.7561454545454</v>
+        <v>563.7440283253591</v>
       </c>
     </row>
     <row r="48">
@@ -2639,13 +2573,13 @@
         <v>5.978989898989899</v>
       </c>
       <c r="M48" t="n">
-        <v>51872.32570505051</v>
+        <v>50184.46889011336</v>
       </c>
       <c r="P48" t="n">
         <v>5.978989898989899</v>
       </c>
       <c r="Q48" t="n">
-        <v>463.2040242424243</v>
+        <v>575.9072924401917</v>
       </c>
     </row>
     <row r="49">
@@ -2665,13 +2599,13 @@
         <v>6.150707070707071</v>
       </c>
       <c r="M49" t="n">
-        <v>54015.25984646466</v>
+        <v>52247.19029813296</v>
       </c>
       <c r="P49" t="n">
         <v>6.150707070707071</v>
       </c>
       <c r="Q49" t="n">
-        <v>472.6519030303031</v>
+        <v>588.0705565550243</v>
       </c>
     </row>
     <row r="50">
@@ -2691,13 +2625,13 @@
         <v>6.322424242424242</v>
       </c>
       <c r="M50" t="n">
-        <v>56158.1939878788</v>
+        <v>54309.91170615256</v>
       </c>
       <c r="P50" t="n">
         <v>6.322424242424242</v>
       </c>
       <c r="Q50" t="n">
-        <v>482.0997818181818</v>
+        <v>600.2338206698568</v>
       </c>
     </row>
     <row r="51">
@@ -2717,13 +2651,13 @@
         <v>6.494141414141414</v>
       </c>
       <c r="M51" t="n">
-        <v>58301.12812929293</v>
+        <v>56372.63311417215</v>
       </c>
       <c r="P51" t="n">
         <v>6.494141414141414</v>
       </c>
       <c r="Q51" t="n">
-        <v>491.5476606060606</v>
+        <v>612.3970847846892</v>
       </c>
     </row>
     <row r="52">
@@ -2743,13 +2677,13 @@
         <v>6.665858585858585</v>
       </c>
       <c r="M52" t="n">
-        <v>60444.06227070707</v>
+        <v>58435.35452219173</v>
       </c>
       <c r="P52" t="n">
         <v>6.665858585858585</v>
       </c>
       <c r="Q52" t="n">
-        <v>500.9955393939393</v>
+        <v>624.5603488995217</v>
       </c>
     </row>
     <row r="53">
@@ -2769,13 +2703,13 @@
         <v>6.837575757575758</v>
       </c>
       <c r="M53" t="n">
-        <v>62586.99641212123</v>
+        <v>60498.07593021134</v>
       </c>
       <c r="P53" t="n">
         <v>6.837575757575758</v>
       </c>
       <c r="Q53" t="n">
-        <v>510.4434181818182</v>
+        <v>636.7236130143544</v>
       </c>
     </row>
     <row r="54">
@@ -2795,13 +2729,13 @@
         <v>7.009292929292929</v>
       </c>
       <c r="M54" t="n">
-        <v>64729.93055353536</v>
+        <v>62560.79733823093</v>
       </c>
       <c r="P54" t="n">
         <v>7.009292929292929</v>
       </c>
       <c r="Q54" t="n">
-        <v>519.891296969697</v>
+        <v>648.8868771291869</v>
       </c>
     </row>
     <row r="55">
@@ -2821,13 +2755,13 @@
         <v>7.1810101010101</v>
       </c>
       <c r="M55" t="n">
-        <v>66872.8646949495</v>
+        <v>64623.51874625053</v>
       </c>
       <c r="P55" t="n">
         <v>7.1810101010101</v>
       </c>
       <c r="Q55" t="n">
-        <v>529.3391757575757</v>
+        <v>661.0501412440194</v>
       </c>
     </row>
     <row r="56">
@@ -2847,13 +2781,13 @@
         <v>7.352727272727273</v>
       </c>
       <c r="M56" t="n">
-        <v>69015.79883636365</v>
+        <v>66686.24015427014</v>
       </c>
       <c r="P56" t="n">
         <v>7.352727272727273</v>
       </c>
       <c r="Q56" t="n">
-        <v>538.7870545454546</v>
+        <v>673.2134053588521</v>
       </c>
     </row>
     <row r="57">
@@ -2873,13 +2807,13 @@
         <v>7.524444444444445</v>
       </c>
       <c r="M57" t="n">
-        <v>71158.73297777779</v>
+        <v>68748.96156228973</v>
       </c>
       <c r="P57" t="n">
         <v>7.524444444444445</v>
       </c>
       <c r="Q57" t="n">
-        <v>548.2349333333334</v>
+        <v>685.3766694736846</v>
       </c>
     </row>
     <row r="58">
@@ -2899,13 +2833,13 @@
         <v>7.696161616161616</v>
       </c>
       <c r="M58" t="n">
-        <v>73301.66711919193</v>
+        <v>70811.68297030931</v>
       </c>
       <c r="P58" t="n">
         <v>7.696161616161616</v>
       </c>
       <c r="Q58" t="n">
-        <v>557.6828121212121</v>
+        <v>697.5399335885171</v>
       </c>
     </row>
     <row r="59">
@@ -2925,13 +2859,13 @@
         <v>7.867878787878787</v>
       </c>
       <c r="M59" t="n">
-        <v>75444.60126060607</v>
+        <v>72874.40437832891</v>
       </c>
       <c r="P59" t="n">
         <v>7.867878787878787</v>
       </c>
       <c r="Q59" t="n">
-        <v>567.1306909090908</v>
+        <v>709.7031977033496</v>
       </c>
     </row>
     <row r="60">
@@ -2951,13 +2885,13 @@
         <v>8.039595959595959</v>
       </c>
       <c r="M60" t="n">
-        <v>77587.53540202019</v>
+        <v>74937.12578634849</v>
       </c>
       <c r="P60" t="n">
         <v>8.039595959595959</v>
       </c>
       <c r="Q60" t="n">
-        <v>576.5785696969697</v>
+        <v>721.8664618181822</v>
       </c>
     </row>
     <row r="61">
@@ -2977,13 +2911,13 @@
         <v>8.211313131313132</v>
       </c>
       <c r="M61" t="n">
-        <v>79730.46954343436</v>
+        <v>76999.84719436811</v>
       </c>
       <c r="P61" t="n">
         <v>8.211313131313132</v>
       </c>
       <c r="Q61" t="n">
-        <v>586.0264484848485</v>
+        <v>734.0297259330148</v>
       </c>
     </row>
     <row r="62">
@@ -3003,13 +2937,13 @@
         <v>8.383030303030303</v>
       </c>
       <c r="M62" t="n">
-        <v>81873.4036848485</v>
+        <v>79062.56860238769</v>
       </c>
       <c r="P62" t="n">
         <v>8.383030303030303</v>
       </c>
       <c r="Q62" t="n">
-        <v>595.4743272727274</v>
+        <v>746.1929900478473</v>
       </c>
     </row>
     <row r="63">
@@ -3029,13 +2963,13 @@
         <v>8.554747474747474</v>
       </c>
       <c r="M63" t="n">
-        <v>84016.33782626262</v>
+        <v>81125.29001040728</v>
       </c>
       <c r="P63" t="n">
         <v>8.554747474747474</v>
       </c>
       <c r="Q63" t="n">
-        <v>604.9222060606061</v>
+        <v>758.3562541626798</v>
       </c>
     </row>
     <row r="64">
@@ -3055,13 +2989,13 @@
         <v>8.726464646464647</v>
       </c>
       <c r="M64" t="n">
-        <v>86159.27196767679</v>
+        <v>83188.01141842689</v>
       </c>
       <c r="P64" t="n">
         <v>8.726464646464647</v>
       </c>
       <c r="Q64" t="n">
-        <v>614.3700848484849</v>
+        <v>770.5195182775125</v>
       </c>
     </row>
     <row r="65">
@@ -3081,13 +3015,13 @@
         <v>8.898181818181818</v>
       </c>
       <c r="M65" t="n">
-        <v>88302.20610909093</v>
+        <v>85250.73282644647</v>
       </c>
       <c r="P65" t="n">
         <v>8.898181818181818</v>
       </c>
       <c r="Q65" t="n">
-        <v>623.8179636363636</v>
+        <v>782.682782392345</v>
       </c>
     </row>
     <row r="66">
@@ -3107,13 +3041,13 @@
         <v>9.06989898989899</v>
       </c>
       <c r="M66" t="n">
-        <v>90445.14025050505</v>
+        <v>87313.45423446607</v>
       </c>
       <c r="P66" t="n">
         <v>9.06989898989899</v>
       </c>
       <c r="Q66" t="n">
-        <v>633.2658424242425</v>
+        <v>794.8460465071774</v>
       </c>
     </row>
     <row r="67">
@@ -3133,13 +3067,13 @@
         <v>9.241616161616161</v>
       </c>
       <c r="M67" t="n">
-        <v>92588.07439191919</v>
+        <v>89376.17564248566</v>
       </c>
       <c r="P67" t="n">
         <v>9.241616161616161</v>
       </c>
       <c r="Q67" t="n">
-        <v>642.7137212121212</v>
+        <v>807.0093106220099</v>
       </c>
     </row>
     <row r="68">
@@ -3159,13 +3093,13 @@
         <v>9.413333333333332</v>
       </c>
       <c r="M68" t="n">
-        <v>94731.00853333333</v>
+        <v>91438.89705050524</v>
       </c>
       <c r="P68" t="n">
         <v>9.413333333333332</v>
       </c>
       <c r="Q68" t="n">
-        <v>652.1616</v>
+        <v>819.1725747368424</v>
       </c>
     </row>
     <row r="69">
@@ -3185,13 +3119,13 @@
         <v>9.585050505050505</v>
       </c>
       <c r="M69" t="n">
-        <v>96873.94267474749</v>
+        <v>93501.61845852486</v>
       </c>
       <c r="P69" t="n">
         <v>9.585050505050505</v>
       </c>
       <c r="Q69" t="n">
-        <v>661.6094787878789</v>
+        <v>831.3358388516751</v>
       </c>
     </row>
     <row r="70">
@@ -3211,13 +3145,13 @@
         <v>9.756767676767677</v>
       </c>
       <c r="M70" t="n">
-        <v>99016.87681616162</v>
+        <v>95564.33986654445</v>
       </c>
       <c r="P70" t="n">
         <v>9.756767676767677</v>
       </c>
       <c r="Q70" t="n">
-        <v>671.0573575757576</v>
+        <v>843.4991029665076</v>
       </c>
     </row>
     <row r="71">
@@ -3237,13 +3171,13 @@
         <v>9.928484848484848</v>
       </c>
       <c r="M71" t="n">
-        <v>101159.8109575758</v>
+        <v>97627.06127456404</v>
       </c>
       <c r="P71" t="n">
         <v>9.928484848484848</v>
       </c>
       <c r="Q71" t="n">
-        <v>680.5052363636364</v>
+        <v>855.6623670813401</v>
       </c>
     </row>
     <row r="72">
@@ -3263,13 +3197,13 @@
         <v>10.10020202020202</v>
       </c>
       <c r="M72" t="n">
-        <v>103302.7450989899</v>
+        <v>99689.78268258365</v>
       </c>
       <c r="P72" t="n">
         <v>10.10020202020202</v>
       </c>
       <c r="Q72" t="n">
-        <v>689.9531151515152</v>
+        <v>867.8256311961728</v>
       </c>
     </row>
     <row r="73">
@@ -3289,13 +3223,13 @@
         <v>10.27191919191919</v>
       </c>
       <c r="M73" t="n">
-        <v>105445.679240404</v>
+        <v>101752.5040906032</v>
       </c>
       <c r="P73" t="n">
         <v>10.27191919191919</v>
       </c>
       <c r="Q73" t="n">
-        <v>699.400993939394</v>
+        <v>879.9888953110053</v>
       </c>
     </row>
     <row r="74">
@@ -3315,13 +3249,13 @@
         <v>10.44363636363636</v>
       </c>
       <c r="M74" t="n">
-        <v>107588.6133818182</v>
+        <v>103815.2254986228</v>
       </c>
       <c r="P74" t="n">
         <v>10.44363636363636</v>
       </c>
       <c r="Q74" t="n">
-        <v>708.8488727272728</v>
+        <v>892.1521594258378</v>
       </c>
     </row>
     <row r="75">
@@ -3341,13 +3275,13 @@
         <v>10.61535353535353</v>
       </c>
       <c r="M75" t="n">
-        <v>109731.5475232323</v>
+        <v>105877.9469066424</v>
       </c>
       <c r="P75" t="n">
         <v>10.61535353535353</v>
       </c>
       <c r="Q75" t="n">
-        <v>718.2967515151515</v>
+        <v>904.3154235406703</v>
       </c>
     </row>
     <row r="76">
@@ -3367,13 +3301,13 @@
         <v>10.78707070707071</v>
       </c>
       <c r="M76" t="n">
-        <v>111874.4816646464</v>
+        <v>107940.668314662</v>
       </c>
       <c r="P76" t="n">
         <v>10.78707070707071</v>
       </c>
       <c r="Q76" t="n">
-        <v>727.7446303030302</v>
+        <v>916.4786876555028</v>
       </c>
     </row>
     <row r="77">
@@ -3393,13 +3327,13 @@
         <v>10.95878787878788</v>
       </c>
       <c r="M77" t="n">
-        <v>114017.4158060606</v>
+        <v>110003.3897226816</v>
       </c>
       <c r="P77" t="n">
         <v>10.95878787878788</v>
       </c>
       <c r="Q77" t="n">
-        <v>737.1925090909092</v>
+        <v>928.6419517703355</v>
       </c>
     </row>
     <row r="78">
@@ -3419,13 +3353,13 @@
         <v>11.13050505050505</v>
       </c>
       <c r="M78" t="n">
-        <v>116160.3499474748</v>
+        <v>112066.1111307012</v>
       </c>
       <c r="P78" t="n">
         <v>11.13050505050505</v>
       </c>
       <c r="Q78" t="n">
-        <v>746.6403878787879</v>
+        <v>940.805215885168</v>
       </c>
     </row>
     <row r="79">
@@ -3445,13 +3379,13 @@
         <v>11.30222222222222</v>
       </c>
       <c r="M79" t="n">
-        <v>118303.2840888889</v>
+        <v>114128.8325387208</v>
       </c>
       <c r="P79" t="n">
         <v>11.30222222222222</v>
       </c>
       <c r="Q79" t="n">
-        <v>756.0882666666666</v>
+        <v>952.9684800000005</v>
       </c>
     </row>
     <row r="80">
@@ -3471,13 +3405,13 @@
         <v>11.47393939393939</v>
       </c>
       <c r="M80" t="n">
-        <v>120446.2182303031</v>
+        <v>116191.5539467404</v>
       </c>
       <c r="P80" t="n">
         <v>11.47393939393939</v>
       </c>
       <c r="Q80" t="n">
-        <v>765.5361454545455</v>
+        <v>965.1317441148332</v>
       </c>
     </row>
     <row r="81">
@@ -3497,13 +3431,13 @@
         <v>11.64565656565657</v>
       </c>
       <c r="M81" t="n">
-        <v>122589.1523717172</v>
+        <v>118254.27535476</v>
       </c>
       <c r="P81" t="n">
         <v>11.64565656565657</v>
       </c>
       <c r="Q81" t="n">
-        <v>774.9840242424243</v>
+        <v>977.2950082296657</v>
       </c>
     </row>
     <row r="82">
@@ -3523,13 +3457,13 @@
         <v>11.81737373737374</v>
       </c>
       <c r="M82" t="n">
-        <v>124732.0865131313</v>
+        <v>120316.9967627796</v>
       </c>
       <c r="P82" t="n">
         <v>11.81737373737374</v>
       </c>
       <c r="Q82" t="n">
-        <v>784.431903030303</v>
+        <v>989.4582723444981</v>
       </c>
     </row>
     <row r="83">
@@ -3549,13 +3483,13 @@
         <v>11.98909090909091</v>
       </c>
       <c r="M83" t="n">
-        <v>126875.0206545455</v>
+        <v>122379.7181707992</v>
       </c>
       <c r="P83" t="n">
         <v>11.98909090909091</v>
       </c>
       <c r="Q83" t="n">
-        <v>793.8797818181819</v>
+        <v>1001.621536459331</v>
       </c>
     </row>
     <row r="84">
@@ -3575,13 +3509,13 @@
         <v>12.16080808080808</v>
       </c>
       <c r="M84" t="n">
-        <v>129017.9547959596</v>
+        <v>124442.4395788188</v>
       </c>
       <c r="P84" t="n">
         <v>12.16080808080808</v>
       </c>
       <c r="Q84" t="n">
-        <v>803.3276606060606</v>
+        <v>1013.784800574163</v>
       </c>
     </row>
     <row r="85">
@@ -3601,13 +3535,13 @@
         <v>12.33252525252525</v>
       </c>
       <c r="M85" t="n">
-        <v>131160.8889373738</v>
+        <v>126505.1609868384</v>
       </c>
       <c r="P85" t="n">
         <v>12.33252525252525</v>
       </c>
       <c r="Q85" t="n">
-        <v>812.7755393939394</v>
+        <v>1025.948064688996</v>
       </c>
     </row>
     <row r="86">
@@ -3627,13 +3561,13 @@
         <v>12.50424242424242</v>
       </c>
       <c r="M86" t="n">
-        <v>133303.8230787879</v>
+        <v>128567.882394858</v>
       </c>
       <c r="P86" t="n">
         <v>12.50424242424242</v>
       </c>
       <c r="Q86" t="n">
-        <v>822.2234181818183</v>
+        <v>1038.111328803828</v>
       </c>
     </row>
     <row r="87">
@@ -3653,13 +3587,13 @@
         <v>12.6759595959596</v>
       </c>
       <c r="M87" t="n">
-        <v>135446.757220202</v>
+        <v>130630.6038028776</v>
       </c>
       <c r="P87" t="n">
         <v>12.6759595959596</v>
       </c>
       <c r="Q87" t="n">
-        <v>831.671296969697</v>
+        <v>1050.274592918661</v>
       </c>
     </row>
     <row r="88">
@@ -3679,13 +3613,13 @@
         <v>12.84767676767677</v>
       </c>
       <c r="M88" t="n">
-        <v>137589.6913616162</v>
+        <v>132693.3252108972</v>
       </c>
       <c r="P88" t="n">
         <v>12.84767676767677</v>
       </c>
       <c r="Q88" t="n">
-        <v>841.1191757575758</v>
+        <v>1062.437857033493</v>
       </c>
     </row>
     <row r="89">
@@ -3705,13 +3639,13 @@
         <v>13.01939393939394</v>
       </c>
       <c r="M89" t="n">
-        <v>139732.6255030303</v>
+        <v>134756.0466189168</v>
       </c>
       <c r="P89" t="n">
         <v>13.01939393939394</v>
       </c>
       <c r="Q89" t="n">
-        <v>850.5670545454547</v>
+        <v>1074.601121148326</v>
       </c>
     </row>
     <row r="90">
@@ -3731,13 +3665,13 @@
         <v>13.19111111111111</v>
       </c>
       <c r="M90" t="n">
-        <v>141875.5596444444</v>
+        <v>136818.7680269364</v>
       </c>
       <c r="P90" t="n">
         <v>13.19111111111111</v>
       </c>
       <c r="Q90" t="n">
-        <v>860.0149333333334</v>
+        <v>1086.764385263158</v>
       </c>
     </row>
     <row r="91">
@@ -3757,13 +3691,13 @@
         <v>13.36282828282828</v>
       </c>
       <c r="M91" t="n">
-        <v>144018.4937858586</v>
+        <v>138881.4894349559</v>
       </c>
       <c r="P91" t="n">
         <v>13.36282828282828</v>
       </c>
       <c r="Q91" t="n">
-        <v>869.4628121212121</v>
+        <v>1098.927649377991</v>
       </c>
     </row>
     <row r="92">
@@ -3783,13 +3717,13 @@
         <v>13.53454545454545</v>
       </c>
       <c r="M92" t="n">
-        <v>146161.4279272727</v>
+        <v>140944.2108429755</v>
       </c>
       <c r="P92" t="n">
         <v>13.53454545454545</v>
       </c>
       <c r="Q92" t="n">
-        <v>878.9106909090909</v>
+        <v>1111.090913492823</v>
       </c>
     </row>
     <row r="93">
@@ -3809,13 +3743,13 @@
         <v>13.70626262626263</v>
       </c>
       <c r="M93" t="n">
-        <v>148304.3620686869</v>
+        <v>143006.9322509951</v>
       </c>
       <c r="P93" t="n">
         <v>13.70626262626263</v>
       </c>
       <c r="Q93" t="n">
-        <v>888.3585696969698</v>
+        <v>1123.254177607656</v>
       </c>
     </row>
     <row r="94">
@@ -3835,13 +3769,13 @@
         <v>13.8779797979798</v>
       </c>
       <c r="M94" t="n">
-        <v>150447.296210101</v>
+        <v>145069.6536590147</v>
       </c>
       <c r="P94" t="n">
         <v>13.8779797979798</v>
       </c>
       <c r="Q94" t="n">
-        <v>897.8064484848485</v>
+        <v>1135.417441722489</v>
       </c>
     </row>
     <row r="95">
@@ -3861,13 +3795,13 @@
         <v>14.04969696969697</v>
       </c>
       <c r="M95" t="n">
-        <v>152590.2303515151</v>
+        <v>147132.3750670343</v>
       </c>
       <c r="P95" t="n">
         <v>14.04969696969697</v>
       </c>
       <c r="Q95" t="n">
-        <v>907.2543272727273</v>
+        <v>1147.580705837321</v>
       </c>
     </row>
     <row r="96">
@@ -3887,13 +3821,13 @@
         <v>14.22141414141414</v>
       </c>
       <c r="M96" t="n">
-        <v>154733.1644929293</v>
+        <v>149195.0964750539</v>
       </c>
       <c r="P96" t="n">
         <v>14.22141414141414</v>
       </c>
       <c r="Q96" t="n">
-        <v>916.7022060606062</v>
+        <v>1159.743969952154</v>
       </c>
     </row>
     <row r="97">
@@ -3913,13 +3847,13 @@
         <v>14.39313131313131</v>
       </c>
       <c r="M97" t="n">
-        <v>156876.0986343434</v>
+        <v>151257.8178830735</v>
       </c>
       <c r="P97" t="n">
         <v>14.39313131313131</v>
       </c>
       <c r="Q97" t="n">
-        <v>926.1500848484848</v>
+        <v>1171.907234066986</v>
       </c>
     </row>
     <row r="98">
@@ -3939,13 +3873,13 @@
         <v>14.56484848484848</v>
       </c>
       <c r="M98" t="n">
-        <v>159019.0327757576</v>
+        <v>153320.5392910931</v>
       </c>
       <c r="P98" t="n">
         <v>14.56484848484848</v>
       </c>
       <c r="Q98" t="n">
-        <v>935.5979636363637</v>
+        <v>1184.070498181819</v>
       </c>
     </row>
     <row r="99">
@@ -3965,13 +3899,13 @@
         <v>14.73656565656566</v>
       </c>
       <c r="M99" t="n">
-        <v>161161.9669171718</v>
+        <v>155383.2606991127</v>
       </c>
       <c r="P99" t="n">
         <v>14.73656565656566</v>
       </c>
       <c r="Q99" t="n">
-        <v>945.0458424242426</v>
+        <v>1196.233762296652</v>
       </c>
     </row>
     <row r="100">
@@ -3991,13 +3925,13 @@
         <v>14.90828282828283</v>
       </c>
       <c r="M100" t="n">
-        <v>163304.9010585858</v>
+        <v>157445.9821071323</v>
       </c>
       <c r="P100" t="n">
         <v>14.90828282828283</v>
       </c>
       <c r="Q100" t="n">
-        <v>954.4937212121212</v>
+        <v>1208.397026411484</v>
       </c>
     </row>
     <row r="101">
@@ -4017,13 +3951,13 @@
         <v>15.08</v>
       </c>
       <c r="M101" t="n">
-        <v>165447.8352</v>
+        <v>159508.7035151519</v>
       </c>
       <c r="P101" t="n">
         <v>15.08</v>
       </c>
       <c r="Q101" t="n">
-        <v>963.9416000000001</v>
+        <v>1220.560290526317</v>
       </c>
     </row>
     <row r="102">

</xml_diff>